<commit_message>
added Lockheed Martin to Ci
</commit_message>
<xml_diff>
--- a/LockheedMartin/lockheed_martin_jobs.xlsx
+++ b/LockheedMartin/lockheed_martin_jobs.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G16"/>
+  <dimension ref="A1:K4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -464,6 +464,26 @@
           <t>General</t>
         </is>
       </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Basic Qualifications</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Desired Skills</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Key responsibilities will include</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -491,8 +511,116 @@
           <t>https://www.lockheedmartinjobs.com/job/king-of-prussia/staff-financial-analyst-ts-clearance/694/84477321856</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr"/>
-      <c r="G2" t="inlineStr"/>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>JOB ID: 700134BR
+Date posted: Jul. 31, 2025
+Description:Space is a critical domain, connecting our technologies, our security and our humanity. While others view space as a destination, we see it as a realm of possibilities, where we can do more— we can innovate, invest, inspire and integrate our capabilities to transform the future. At Lockheed Martin Space, we aim to harness the full potential of space to cultivate innovation, reduce costs, and push the boundaries of what technology can achieve. We’re creating future-ready solutions, focusing on resiliency and urgency through our 21st Century Security® vision. We’re erasing boundaries and forming partnerships across industries and around the world. We’re advancing spacecraft and the workforce to fuel the next generation. And we’re reimagining how space can connect us, ensuring security and prosperity. Join us in shaping a new era in space and find a career that's built for you.
+Selected candidate will perform as lead Program Finance/Program Accounting analyst on Stormbreaker contract.
+Will be responsible for leading financial support and analyses, but not limited to, to following:
+Establish and monitor program budgets
+• Track and reconcile costs, highlighting issues/concerns/trends to the program team
+• Track program funding requirements and prepare monthly Contract Funds Status Reports (CFSRs) for each Task Order
+• Conduct cost analyses and develop variance explanations with recommendations for corrective actions as required
+• Prepare quarterly Estimates to Complete (EACs) and Contract Status Reports (CSRs)
+• Coordinate and prepare monthly financial reviews with Functional Area Management
+• Other financial support as required (e.g. billing coordination, AP and cash coordination/reporting/tracking, etc.)
+• Needs to be able to maintain a TS/ SCI clearance in this role
+Basic Qualifications:
+- Bachelors or Masters or higher level degree
+- Proven analytical ability
+- Working knowledge of various Finance functions (i.e. EVM or contracts or estimating or planning or finance analyst or FP&amp;A, or anything else related.)
+- Experience with Microsoft Office products
+- Active TS clearance
+Desired Skills:
+- Ability to multi-task, prioritize work, and manage multiple deadlines in dynamic environment
+- Demonstrated ability to Analyze &amp; Interpret complex Program Metrics
+- Solid written and verbal communication skills
+- Quick learner with aptitude for various systems and processes
+- Proved work style focusing on accountability and professionalism
+- Experience developing presentation packages and presenting to senior leadership
+- Works effectively as an individual contributor and as part of a team
+- Bachelors degree from an accredited college in a related discipline, or equivalent experience/combined education, with 10+ years of professional experience; or 8+ years of professional experience with a related Masters degree.
+- TS/ SCI clearance
+Security Clearance Statement:This position requires a government security clearance, you must be a US Citizen for consideration.
+Clearance Level:TS/SCI
+Other Important Information You Should Know
+Expression of Interest:By applying to this job, you are expressing interest in this position and could be considered for other career opportunities where similar skills and requirements have been identified as a match. Should this match be identified you may be contacted for this and future openings.
+Ability to Work Remotely:Onsite Full-time: The work associated with this position will be performed onsite at a designated Lockheed Martin facility.
+Work Schedules:Lockheed Martin supports a variety of alternate work schedules that provide additional flexibility to our employees. Schedules range from standard 40 hours over a five day work week while others may be condensed. These condensed schedules provide employees with additional time away from the office and are in addition to our Paid Time off benefits.
+Schedule for this Position:9x80 every other Friday off
+Lockheed Martin is an equal opportunity employer. Qualified candidates will be considered without regard to legally protected characteristics.
+The application window will close in 90 days; applicants are encouraged to apply within 5 - 30 days of the requisition posting date in order to receive optimal consideration.
+At Lockheed Martin, we use our passion for purposeful innovation to help keep people safe and solve the world's most complex challenges. Our people are some of the greatest minds in the industry and truly make Lockheed Martin a great place to work.
+With our employees as our priority, we provide diverse career opportunities designed to propel, develop, and boost agility. Our flexible schedules, competitive pay, and comprehensive benefits enable our employees to live a healthy, fulfilling life at and outside of work. We place an emphasis on empowering our employees by fostering an inclusive environment built upon integrity and corporate responsibility.
+If this sounds like a culture you connect with, you’re invited to apply for this role. Or, if you are unsure whether your experience aligns with the requirements of this position, we encourage you to search on Lockheed Martin Jobs, and apply for roles that align with your qualifications.
+Experience Level:Experienced Professional
+Business Unit:SPACE
+Relocation Available:Possible
+Career Area:Finance
+Type:Full-Time
+Shift:First</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>JOB ID: 700134BR
+Date posted: Jul. 31, 2025
+Description:Space is a critical domain, connecting our technologies, our security and our humanity. While others view space as a destination, we see it as a realm of possibilities, where we can do more— we can innovate, invest, inspire and integrate our capabilities to transform the future. At Lockheed Martin Space, we aim to harness the full potential of space to cultivate innovation, reduce costs, and push the boundaries of what technology can achieve. We’re creating future-ready solutions, focusing on resiliency and urgency through our 21st Century Security® vision. We’re erasing boundaries and forming partnerships across industries and around the world. We’re advancing spacecraft and the workforce to fuel the next generation. And we’re reimagining how space can connect us, ensuring security and prosperity. Join us in shaping a new era in space and find a career that's built for you.
+Selected candidate will perform as lead Program Finance/Program Accounting analyst on Stormbreaker contract.
+Will be responsible for leading financial support and analyses, but not limited to, to following:
+Establish and monitor program budgets
+• Track and reconcile costs, highlighting issues/concerns/trends to the program team
+• Track program funding requirements and prepare monthly Contract Funds Status Reports (CFSRs) for each Task Order
+• Conduct cost analyses and develop variance explanations with recommendations for corrective actions as required
+• Prepare quarterly Estimates to Complete (EACs) and Contract Status Reports (CSRs)
+• Coordinate and prepare monthly financial reviews with Functional Area Management
+• Other financial support as required (e.g. billing coordination, AP and cash coordination/reporting/tracking, etc.)
+• Needs to be able to maintain a TS/ SCI clearance in this role</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>- Bachelors or Masters or higher level degree
+- Proven analytical ability
+- Working knowledge of various Finance functions (i.e. EVM or contracts or estimating or planning or finance analyst or FP&amp;A, or anything else related.)
+- Experience with Microsoft Office products
+- Active TS clearance</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>- Ability to multi-task, prioritize work, and manage multiple deadlines in dynamic environment
+- Demonstrated ability to Analyze &amp; Interpret complex Program Metrics
+- Solid written and verbal communication skills
+- Quick learner with aptitude for various systems and processes
+- Proved work style focusing on accountability and professionalism
+- Experience developing presentation packages and presenting to senior leadership
+- Works effectively as an individual contributor and as part of a team
+- Bachelors degree from an accredited college in a related discipline, or equivalent experience/combined education, with 10+ years of professional experience; or 8+ years of professional experience with a related Masters degree.
+- TS/ SCI clearance
+Security Clearance Statement:This position requires a government security clearance, you must be a US Citizen for consideration.
+Clearance Level:TS/SCI
+Other Important Information You Should Know
+Expression of Interest:By applying to this job, you are expressing interest in this position and could be considered for other career opportunities where similar skills and requirements have been identified as a match. Should this match be identified you may be contacted for this and future openings.
+Ability to Work Remotely:Onsite Full-time: The work associated with this position will be performed onsite at a designated Lockheed Martin facility.
+Work Schedules:Lockheed Martin supports a variety of alternate work schedules that provide additional flexibility to our employees. Schedules range from standard 40 hours over a five day work week while others may be condensed. These condensed schedules provide employees with additional time away from the office and are in addition to our Paid Time off benefits.
+Schedule for this Position:9x80 every other Friday off
+Lockheed Martin is an equal opportunity employer. Qualified candidates will be considered without regard to legally protected characteristics.
+The application window will close in 90 days; applicants are encouraged to apply within 5 - 30 days of the requisition posting date in order to receive optimal consideration.
+At Lockheed Martin, we use our passion for purposeful innovation to help keep people safe and solve the world's most complex challenges. Our people are some of the greatest minds in the industry and truly make Lockheed Martin a great place to work.
+With our employees as our priority, we provide diverse career opportunities designed to propel, develop, and boost agility. Our flexible schedules, competitive pay, and comprehensive benefits enable our employees to live a healthy, fulfilling life at and outside of work. We place an emphasis on empowering our employees by fostering an inclusive environment built upon integrity and corporate responsibility.
+If this sounds like a culture you connect with, you’re invited to apply for this role. Or, if you are unsure whether your experience aligns with the requirements of this position, we encourage you to search on Lockheed Martin Jobs, and apply for roles that align with your qualifications.
+Experience Level:Experienced Professional
+Business Unit:SPACE
+Relocation Available:Possible
+Career Area:Finance
+Type:Full-Time
+Shift:First</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr"/>
+      <c r="K2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -520,8 +648,128 @@
           <t>https://www.lockheedmartinjobs.com/job/orlando/data-scientist-analyst-senior-orlando-fl/694/84477320672</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr"/>
-      <c r="G3" t="inlineStr"/>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>JOB ID: 699865BR
+Date posted: Jul. 31, 2025
+Description:
+Lockheed Martin is a global security and aerospace company that employs approximately 114,000 people worldwide and is principally engaged in the research, design, development, manufacture, integration and sustainment of advanced technology systems, products and services. Lockheed Martin Missiles and Fire Control (MFC) is one of four Lockheed Martin business areas. MFC is a recognized designer, developer and manufacturer of precision engagement aerospace and defense systems for the U.S. and allied militaries. MFC develops, manufactures and supports advanced products for military customers that include the U.S. Army, Navy, Air Force, Marine Corps, NASA and dozens of foreign allies. MFC also offers a wide range of products and services for the global civil nuclear power industry and the military’s green power initiatives.
+What You Will Be Doing
+The successful candidate will leverage advanced analytics, statistical modeling, and machine learning to drive data-driven decision-making across MFC engineering and production. You will apply advanced statistical techniques, machine learning algorithms, and data visualization methods to identify trends, patterns, and correlations in data from engineering development and production sources. You will develop, implement, and advocate for AI-powered solutions.
+Key responsibilities will include:
+• Data wrangling and curation: extracting, transforming, and loading data from various sources, including legacy databases, SAP products, and other enterprise systems.
+• ETL (Extract, Transform, Load) process development and optimization: designing and implementing efficient data pipelines to support data analytics and machine learning workflows.
+• Data quality and integrity: ensuring data accuracy, completeness, and consistency, and developing processes to monitor and maintain data quality over time.
+• Data governance: working with stakeholders to develop and implement data governance policies and procedures, including data security, compliance, and privacy regulations.
+• Data storytelling: using data visualization and communication techniques to translate complex data insights and recommendations to non-technical stakeholders and leadership.
+Why Join Us
+Do you want to be part of a company culture that encourages employees to build their career, leverage their knowledge while using cutting edge technology, and achieve challenging goals? We provide the foundation and resources to help you stay motivated, inspired, and productive. If you are driven, dedicated, and enjoy doing what you love, then we want you to join our journey and build a better tomorrow with you.
+We offer flexible work schedules to comprehensive benefits investing in your future and security, Learn more about Lockheed Martin’s comprehensive benefits package here.
+Basic Qualifications:
+• Bachelor’s degree in Data Science, Mathematics, Statistics, or Computer Science.
+• Experience in data analysis, including data wrangling, curation, and engineering.
+• Strong understanding of database concepts, including data modeling, database design, and query optimization.
+• Experience with SQL, including complex query writing and optimization.
+• Experience working with legacy databases, including data migration, integration, and optimization.
+• Familiarity with products from SAP, including ERP, CRM, and data analytics tools.
+• Strong programming skill in python.
+• BI tools expertise
+• Data visualization experience
+• SAP Business Objects experience
+• Ability to obtain a secret security clearance and therefore must be US Citizen.
+Desired Skills:
+• 5+ years experience working and leading Data Science based projects.
+• Proficiency with containerization technologies, such as Docker and Kubernetes.
+• Strong understanding of statistical modeling and machine learning techniques.
+• Experience in deployment of AI and statistical algorithm systems on high performance compute infrastructure.
+Security Clearance Statement: This position requires a government security clearance, you must be a US Citizen for consideration.
+Clearance Level: Secret
+Other Important Information You Should Know
+Expression of Interest: By applying to this job, you are expressing interest in this position and could be considered for other career opportunities where similar skills and requirements have been identified as a match. Should this match be identified you may be contacted for this and future openings.
+Ability to Work Remotely: Full-time Remote Telework: The employee selected for this position will work remotely full time at a location other than a Lockheed Martin designated office/job site. Employees may travel to a Lockheed Martin office for periodic meetings.
+Work Schedules: Lockheed Martin supports a variety of alternate work schedules that provide additional flexibility to our employees. Schedules range from standard 40 hours over a five day work week while others may be condensed. These condensed schedules provide employees with additional time away from the office and are in addition to our Paid Time off benefits.
+Schedule for this Position: 4x10 hour day, 3 days off per week
+Pay Rate: The annual base salary range for this position in most major metropolitan areas in California and New York is $111,700 - $193,660. For states not referenced above, the salary range for this position will reflect the candidate’s final work location. Please note that the salary information is a general guideline only. Lockheed Martin considers factors such as (but not limited to) scope and responsibilities of the position, candidate's work experience, education/ training, key skills as well as market and business considerations when extending an offer. Benefits offered: Medical, Dental, Vision, Life Insurance, Short-Term Disability, Long-Term Disability, 401(k) match, Flexible Spending Accounts, EAP, Education Assistance, Parental Leave, Paid time off, and Holidays. This position is incentive plan eligible.
+Pay Rate: The annual base salary range for this position in California and New York (excluding most major metropolitan areas), Colorado, Hawaii, Illinois, Maryland, Minnesota, New Jersey, Vermont, Washington or Washington DC is $97,100 - $171,235. For states not referenced above, the salary range for this position will reflect the candidate’s final work location. Please note that the salary information is a general guideline only. Lockheed Martin considers factors such as (but not limited to) scope and responsibilities of the position, candidate's work experience, education/ training, key skills as well as market and business considerations when extending an offer. Benefits offered: Medical, Dental, Vision, Life Insurance, Short-Term Disability, Long-Term Disability, 401(k) match, Flexible Spending Accounts, EAP, Education Assistance, Parental Leave, Paid time off, and Holidays. (Washington state applicants only) Non-represented full-time employees: accrue at least 10 hours per month of Paid Time Off (PTO) to be used for incidental absences and other reasons; receive at least 90 hours for holidays. Represented full time employees accrue 6.67 hours of Vacation per month; accrue up to 52 hours of sick leave annually; receive at least 96 hours for holidays. PTO, Vacation, sick leave, and holiday hours are prorated based on start date during the calendar year. This position is incentive plan eligible.
+Lockheed Martin is an equal opportunity employer. Qualified candidates will be considered without regard to legally protected characteristics.
+The application window will close in 90 days; applicants are encouraged to apply within 5 - 30 days of the requisition posting date in order to receive optimal consideration.
+Join us at Lockheed Martin, where your mission is ours. Our customers tackle the hardest missions. Those that demand extraordinary amounts of courage, resilience and precision. They’re dangerous. Critical. Sometimes they even provide an opportunity to change the world and save lives. Those are the missions we care about.
+As a leading technology innovation company, Lockheed Martin’s vast team works with partners around the world to bring proven performance to our customers’ toughest challenges. Lockheed Martin has employees based in many states throughout the U.S., and Internationally, with business locations in many nations and territories.
+Experience Level: Experienced Professional
+Business Unit: MISSILES AND FIRE CONTROL
+Relocation Available: No
+Career Area: Software Engineering
+Type: Full-Time
+Shift: First</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>JOB ID: 699865BR
+Date posted: Jul. 31, 2025</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>• Bachelor’s degree in Data Science, Mathematics, Statistics, or Computer Science.
+• Experience in data analysis, including data wrangling, curation, and engineering.
+• Strong understanding of database concepts, including data modeling, database design, and query optimization.
+• Experience with SQL, including complex query writing and optimization.
+• Experience working with legacy databases, including data migration, integration, and optimization.
+• Familiarity with products from SAP, including ERP, CRM, and data analytics tools.
+• Strong programming skill in python.
+• BI tools expertise
+• Data visualization experience
+• SAP Business Objects experience
+• Ability to obtain a secret security clearance and therefore must be US Citizen.</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>• 5+ years experience working and leading Data Science based projects.
+• Proficiency with containerization technologies, such as Docker and Kubernetes.
+• Strong understanding of statistical modeling and machine learning techniques.
+• Experience in deployment of AI and statistical algorithm systems on high performance compute infrastructure.
+Security Clearance Statement: This position requires a government security clearance, you must be a US Citizen for consideration.
+Clearance Level: Secret
+Other Important Information You Should Know
+Expression of Interest: By applying to this job, you are expressing interest in this position and could be considered for other career opportunities where similar skills and requirements have been identified as a match. Should this match be identified you may be contacted for this and future openings.
+Ability to Work Remotely: Full-time Remote Telework: The employee selected for this position will work remotely full time at a location other than a Lockheed Martin designated office/job site. Employees may travel to a Lockheed Martin office for periodic meetings.
+Work Schedules: Lockheed Martin supports a variety of alternate work schedules that provide additional flexibility to our employees. Schedules range from standard 40 hours over a five day work week while others may be condensed. These condensed schedules provide employees with additional time away from the office and are in addition to our Paid Time off benefits.
+Schedule for this Position: 4x10 hour day, 3 days off per week
+Pay Rate: The annual base salary range for this position in most major metropolitan areas in California and New York is $111,700 - $193,660. For states not referenced above, the salary range for this position will reflect the candidate’s final work location. Please note that the salary information is a general guideline only. Lockheed Martin considers factors such as (but not limited to) scope and responsibilities of the position, candidate's work experience, education/ training, key skills as well as market and business considerations when extending an offer. Benefits offered: Medical, Dental, Vision, Life Insurance, Short-Term Disability, Long-Term Disability, 401(k) match, Flexible Spending Accounts, EAP, Education Assistance, Parental Leave, Paid time off, and Holidays. This position is incentive plan eligible.
+Pay Rate: The annual base salary range for this position in California and New York (excluding most major metropolitan areas), Colorado, Hawaii, Illinois, Maryland, Minnesota, New Jersey, Vermont, Washington or Washington DC is $97,100 - $171,235. For states not referenced above, the salary range for this position will reflect the candidate’s final work location. Please note that the salary information is a general guideline only. Lockheed Martin considers factors such as (but not limited to) scope and responsibilities of the position, candidate's work experience, education/ training, key skills as well as market and business considerations when extending an offer. Benefits offered: Medical, Dental, Vision, Life Insurance, Short-Term Disability, Long-Term Disability, 401(k) match, Flexible Spending Accounts, EAP, Education Assistance, Parental Leave, Paid time off, and Holidays. (Washington state applicants only) Non-represented full-time employees: accrue at least 10 hours per month of Paid Time Off (PTO) to be used for incidental absences and other reasons; receive at least 90 hours for holidays. Represented full time employees accrue 6.67 hours of Vacation per month; accrue up to 52 hours of sick leave annually; receive at least 96 hours for holidays. PTO, Vacation, sick leave, and holiday hours are prorated based on start date during the calendar year. This position is incentive plan eligible.
+Lockheed Martin is an equal opportunity employer. Qualified candidates will be considered without regard to legally protected characteristics.
+The application window will close in 90 days; applicants are encouraged to apply within 5 - 30 days of the requisition posting date in order to receive optimal consideration.
+Join us at Lockheed Martin, where your mission is ours. Our customers tackle the hardest missions. Those that demand extraordinary amounts of courage, resilience and precision. They’re dangerous. Critical. Sometimes they even provide an opportunity to change the world and save lives. Those are the missions we care about.
+As a leading technology innovation company, Lockheed Martin’s vast team works with partners around the world to bring proven performance to our customers’ toughest challenges. Lockheed Martin has employees based in many states throughout the U.S., and Internationally, with business locations in many nations and territories.
+Experience Level: Experienced Professional
+Business Unit: MISSILES AND FIRE CONTROL
+Relocation Available: No
+Career Area: Software Engineering
+Type: Full-Time
+Shift: First</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>Lockheed Martin is a global security and aerospace company that employs approximately 114,000 people worldwide and is principally engaged in the research, design, development, manufacture, integration and sustainment of advanced technology systems, products and services. Lockheed Martin Missiles and Fire Control (MFC) is one of four Lockheed Martin business areas. MFC is a recognized designer, developer and manufacturer of precision engagement aerospace and defense systems for the U.S. and allied militaries. MFC develops, manufactures and supports advanced products for military customers that include the U.S. Army, Navy, Air Force, Marine Corps, NASA and dozens of foreign allies. MFC also offers a wide range of products and services for the global civil nuclear power industry and the military’s green power initiatives.
+What You Will Be Doing
+The successful candidate will leverage advanced analytics, statistical modeling, and machine learning to drive data-driven decision-making across MFC engineering and production. You will apply advanced statistical techniques, machine learning algorithms, and data visualization methods to identify trends, patterns, and correlations in data from engineering development and production sources. You will develop, implement, and advocate for AI-powered solutions.</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>• Data wrangling and curation: extracting, transforming, and loading data from various sources, including legacy databases, SAP products, and other enterprise systems.
+• ETL (Extract, Transform, Load) process development and optimization: designing and implementing efficient data pipelines to support data analytics and machine learning workflows.
+• Data quality and integrity: ensuring data accuracy, completeness, and consistency, and developing processes to monitor and maintain data quality over time.
+• Data governance: working with stakeholders to develop and implement data governance policies and procedures, including data security, compliance, and privacy regulations.
+• Data storytelling: using data visualization and communication techniques to translate complex data insights and recommendations to non-technical stakeholders and leadership.
+Why Join Us
+Do you want to be part of a company culture that encourages employees to build their career, leverage their knowledge while using cutting edge technology, and achieve challenging goals? We provide the foundation and resources to help you stay motivated, inspired, and productive. If you are driven, dedicated, and enjoy doing what you love, then we want you to join our journey and build a better tomorrow with you.
+We offer flexible work schedules to comprehensive benefits investing in your future and security, Learn more about Lockheed Martin’s comprehensive benefits package here.</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -549,356 +797,128 @@
           <t>https://www.lockheedmartinjobs.com/job/littleton/senior-industrial-engineer/694/84477319024</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr"/>
-      <c r="G4" t="inlineStr"/>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Manufacturing Materials Resource Planner - Entry level</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>84477317568</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>Date Posted: 07/30/2025</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>Littleton, Colorado</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>https://www.lockheedmartinjobs.com/job/littleton/manufacturing-materials-resource-planner-entry-level/694/84477317568</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr"/>
-      <c r="G5" t="inlineStr"/>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Multi Function Manufacturing Planner Associate Manager</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>84477317152</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>Date Posted: 07/30/2025</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>Meridian, Mississippi</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>https://www.lockheedmartinjobs.com/job/meridian/multi-function-manufacturing-planner-associate-manager/694/84477317152</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr"/>
-      <c r="G6" t="inlineStr"/>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>Land and Maritime Solutions Business Development Director</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>81893086032</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>Date Posted: 07/23/2025</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>Orlando, Florida</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>https://www.lockheedmartinjobs.com/job/orlando/land-and-maritime-solutions-business-development-director/694/81893086032</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr"/>
-      <c r="G7" t="inlineStr"/>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>Principal Circuit Design Engineer, Avionics Development</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>84472661120</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>Date Posted: 07/30/2025</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>Littleton, Colorado</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>https://www.lockheedmartinjobs.com/job/littleton/principal-circuit-design-engineer-avionics-development/694/84472661120</t>
-        </is>
-      </c>
-      <c r="F8" t="inlineStr"/>
-      <c r="G8" t="inlineStr"/>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>Information Systems Admin (Level 4) Mission Planning, NAS Fallon</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>84472660896</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>Date Posted: 07/30/2025</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>Fallon, Nevada</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>https://www.lockheedmartinjobs.com/job/fallon/information-systems-admin-level-4-mission-planning-nas-fallon/694/84472660896</t>
-        </is>
-      </c>
-      <c r="F9" t="inlineStr"/>
-      <c r="G9" t="inlineStr"/>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>Electronics Engineer III, Missile Avionics</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>84472660640</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>Date Posted: 07/30/2025</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>Sunnyvale, California</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>https://www.lockheedmartinjobs.com/job/sunnyvale/electronics-engineer-iii-missile-avionics/694/84472660640</t>
-        </is>
-      </c>
-      <c r="F10" t="inlineStr"/>
-      <c r="G10" t="inlineStr"/>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>Electronics Engineer III, Missile Avionics</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>84472660464</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>Date Posted: 07/30/2025</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>Sunnyvale, California</t>
-        </is>
-      </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>https://www.lockheedmartinjobs.com/job/sunnyvale/electronics-engineer-iii-missile-avionics/694/84472660464</t>
-        </is>
-      </c>
-      <c r="F11" t="inlineStr"/>
-      <c r="G11" t="inlineStr"/>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>Software Engineer (SWE2) with Poly Mid to SR</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>84472660064</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>Date Posted: 07/30/2025</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>Annapolis Junction, Maryland</t>
-        </is>
-      </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>https://www.lockheedmartinjobs.com/job/annapolis-junction/software-engineer-swe2-with-poly-mid-to-sr/694/84472660064</t>
-        </is>
-      </c>
-      <c r="F12" t="inlineStr"/>
-      <c r="G12" t="inlineStr"/>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>Software Engineer With Poly Early to Mid</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>84472659536</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>Date Posted: 07/30/2025</t>
-        </is>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>Annapolis Junction, Maryland</t>
-        </is>
-      </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>https://www.lockheedmartinjobs.com/job/annapolis-junction/software-engineer-with-poly-early-to-mid/694/84472659536</t>
-        </is>
-      </c>
-      <c r="F13" t="inlineStr"/>
-      <c r="G13" t="inlineStr"/>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>Software Engineer With Poly Early to Mid</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>84472659120</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>Date Posted: 07/30/2025</t>
-        </is>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>Annapolis Junction, Maryland</t>
-        </is>
-      </c>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>https://www.lockheedmartinjobs.com/job/annapolis-junction/software-engineer-with-poly-early-to-mid/694/84472659120</t>
-        </is>
-      </c>
-      <c r="F14" t="inlineStr"/>
-      <c r="G14" t="inlineStr"/>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>DevSecOps Computational Engineer / Onsite - Orlando, FL</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>84472653792</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>Date Posted: 07/30/2025</t>
-        </is>
-      </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>Orlando, Florida</t>
-        </is>
-      </c>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>https://www.lockheedmartinjobs.com/job/orlando/devsecops-computational-engineer-onsite-orlando-fl/694/84472653792</t>
-        </is>
-      </c>
-      <c r="F15" t="inlineStr"/>
-      <c r="G15" t="inlineStr"/>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>GNC Modeling &amp; Simulation Staff Engineer - Grand Prairie, TX</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>84472648608</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>Date Posted: 07/30/2025</t>
-        </is>
-      </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>Grand Prairie, Texas</t>
-        </is>
-      </c>
-      <c r="E16" t="inlineStr">
-        <is>
-          <t>https://www.lockheedmartinjobs.com/job/grand-prairie/gnc-modeling-and-simulation-staff-engineer-grand-prairie-tx/694/84472648608</t>
-        </is>
-      </c>
-      <c r="F16" t="inlineStr"/>
-      <c r="G16" t="inlineStr"/>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>JOB ID: 699634BR
+Date posted: Jul. 31, 2025
+Description:Lockheed Martin Space is seeking a Senior Industrial Engineer to join our team in Littleton, CO!
+The Industrial Engineering team is known for delivering breakthrough capabilities and process improvement that continually redefine space flight. As our business grows, we are looking to expand our industrial engineering team with someone who can help us deliver breakthrough capabilities that redefine our production systems. This talented team understands data and loves building tools that use data to surface problems and give people a convenient way to act. Industrial Engineers operate in a fast-paced, agile, next-gen environment, and utilize the latest technology in PLM, MRP, MES, Discrete Event Simulation, Data Analytics, and Data Visualization Software to produce analysis’ &amp; metrics which enable imperative business decisions.
+If you possess a passion for continuous improvement and are always looking for ways to reduce waste, improve human factors, and introduce technology to effect change, this may be the role for you!
+This is an experienced Industrial Engineering opportunity where you will:
+• Apply advanced Industrial Engineering concepts and techniques to analyze business processes and reduce waste.
+• Working with facilities engineers to support planning of new production lines and factories.
+• Supporting Manufacturing Engineers in developing standards and analyzing shop performance against targets.
+• Generating production process simulations for future production programs and performing analyses to identify resource constraints, flow, process layouts, and work schedules to achieve delivery targets.
+• Interrogate data systems and look for opportunities to surface problems and drive improvements.
+• Oversee process improvement efforts, ensuring implementation and sustainment while demonstrating results.
+• Mentor, lead, and train less experienced industrial engineers
+• Supporting occasional weekend or off-hour support as needed to maintain production schedule compliance.
+• Interact with shop floor production operations team to enable the IE to comprehend the manufacturing processes to provide data-driven deliverables to internal customers.
+• Collaborate with all functional groups through the entire product lifecycle within a production environment
+• Provide valuable solutions to multiple organizations and align program priorities.
+Basic Qualifications:
+• Industrial Engineering experience in manufacturing
+• Project management experience
+• Experience developing, monitoring and/or reporting metrics related to cost and schedule performance specific to standard cost
+• Experience developing forecasts and/or Production Schedules and/or Resource Load Staffing Plans
+• Experience with discrete event simulation of production processes
+• Must be able to obtain and maintain Top Secret clearance
+Desired Skills:
+• Bachelor's degree or higher education from an accredited college or equivalent experience
+•Experience with standing up new production manufacturing lines / factories
+•Leadership experience. Proven ability to maintain a high performing team. Ability to manage and resolve conflict.
+•Experience with SAP, Apriso, VECAMS, Tableau, Simio or other simulation software
+• Excellent communication skills (verbal, written and presentation), particularly with Production Operations and Program Offices
+• Ability to multi-task, organize and prioritize assignments
+• Production Experience and/or New Production Program Experience
+• Ability to construct PowerPoint presentation material and brief to senior leadership effectively
+• Active Top Secret security clearance
+Security Clearance Statement:This position requires a government security clearance, you must be a US Citizen for consideration.
+Clearance Level:Top Secret
+Other Important Information You Should Know
+Expression of Interest:By applying to this job, you are expressing interest in this position and could be considered for other career opportunities where similar skills and requirements have been identified as a match. Should this match be identified you may be contacted for this and future openings.
+Ability to Work Remotely:Onsite Full-time: The work associated with this position will be performed onsite at a designated Lockheed Martin facility.
+Work Schedules:Lockheed Martin supports a variety of alternate work schedules that provide additional flexibility to our employees. Schedules range from standard 40 hours over a five day work week while others may be condensed. These condensed schedules provide employees with additional time away from the office and are in addition to our Paid Time off benefits.
+Schedule for this Position:9x80 every other Friday off
+Pay Rate: The annual base salary range for this position in California and New York (excluding most major metropolitan areas), Colorado, Hawaii, Illinois, Maryland, Minnesota, New Jersey, Vermont, Washington or Washington DC is $77,700 - $136,965. For states not referenced above, the salary range for this position will reflect the candidate’s final work location. Please note that the salary information is a general guideline only. Lockheed Martin considers factors such as (but not limited to) scope and responsibilities of the position, candidate's work experience, education/ training, key skills as well as market and business considerations when extending an offer. Benefits offered: Medical, Dental, Vision, Life Insurance, Short-Term Disability, Long-Term Disability, 401(k) match, Flexible Spending Accounts, EAP, Education Assistance, Parental Leave, Paid time off, and Holidays. (Washington state applicants only) Non-represented full-time employees: accrue at least 10 hours per month of Paid Time Off (PTO) to be used for incidental absences and other reasons; receive at least 90 hours for holidays. Represented full time employees accrue 6.67 hours of Vacation per month; accrue up to 52 hours of sick leave annually; receive at least 96 hours for holidays. PTO, Vacation, sick leave, and holiday hours are prorated based on start date during the calendar year. This position is incentive plan eligible.
+Lockheed Martin is an equal opportunity employer. Qualified candidates will be considered without regard to legally protected characteristics.
+The application window will close in 90 days; applicants are encouraged to apply within 5 - 30 days of the requisition posting date in order to receive optimal consideration.
+At Lockheed Martin, we use our passion for purposeful innovation to help keep people safe and solve the world's most complex challenges. Our people are some of the greatest minds in the industry and truly make Lockheed Martin a great place to work.
+With our employees as our priority, we provide diverse career opportunities designed to propel, develop, and boost agility. Our flexible schedules, competitive pay, and comprehensive benefits enable our employees to live a healthy, fulfilling life at and outside of work. We place an emphasis on empowering our employees by fostering an inclusive environment built upon integrity and corporate responsibility.
+If this sounds like a culture you connect with, you’re invited to apply for this role. Or, if you are unsure whether your experience aligns with the requirements of this position, we encourage you to search on Lockheed Martin Jobs, and apply for roles that align with your qualifications.
+Experience Level:Experienced Professional
+Business Unit:SPACE
+Relocation Available:Possible
+Career Area:Manufacturing
+Type:Full-Time
+Shift:First</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>JOB ID: 699634BR
+Date posted: Jul. 31, 2025
+Description:Lockheed Martin Space is seeking a Senior Industrial Engineer to join our team in Littleton, CO!
+The Industrial Engineering team is known for delivering breakthrough capabilities and process improvement that continually redefine space flight. As our business grows, we are looking to expand our industrial engineering team with someone who can help us deliver breakthrough capabilities that redefine our production systems. This talented team understands data and loves building tools that use data to surface problems and give people a convenient way to act. Industrial Engineers operate in a fast-paced, agile, next-gen environment, and utilize the latest technology in PLM, MRP, MES, Discrete Event Simulation, Data Analytics, and Data Visualization Software to produce analysis’ &amp; metrics which enable imperative business decisions.
+If you possess a passion for continuous improvement and are always looking for ways to reduce waste, improve human factors, and introduce technology to effect change, this may be the role for you!
+This is an experienced Industrial Engineering opportunity where you will:
+• Apply advanced Industrial Engineering concepts and techniques to analyze business processes and reduce waste.
+• Working with facilities engineers to support planning of new production lines and factories.
+• Supporting Manufacturing Engineers in developing standards and analyzing shop performance against targets.
+• Generating production process simulations for future production programs and performing analyses to identify resource constraints, flow, process layouts, and work schedules to achieve delivery targets.
+• Interrogate data systems and look for opportunities to surface problems and drive improvements.
+• Oversee process improvement efforts, ensuring implementation and sustainment while demonstrating results.
+• Mentor, lead, and train less experienced industrial engineers
+• Supporting occasional weekend or off-hour support as needed to maintain production schedule compliance.
+• Interact with shop floor production operations team to enable the IE to comprehend the manufacturing processes to provide data-driven deliverables to internal customers.
+• Collaborate with all functional groups through the entire product lifecycle within a production environment
+• Provide valuable solutions to multiple organizations and align program priorities.</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>• Industrial Engineering experience in manufacturing
+• Project management experience
+• Experience developing, monitoring and/or reporting metrics related to cost and schedule performance specific to standard cost
+• Experience developing forecasts and/or Production Schedules and/or Resource Load Staffing Plans
+• Experience with discrete event simulation of production processes
+• Must be able to obtain and maintain Top Secret clearance</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>• Bachelor's degree or higher education from an accredited college or equivalent experience
+•Experience with standing up new production manufacturing lines / factories
+•Leadership experience. Proven ability to maintain a high performing team. Ability to manage and resolve conflict.
+•Experience with SAP, Apriso, VECAMS, Tableau, Simio or other simulation software
+• Excellent communication skills (verbal, written and presentation), particularly with Production Operations and Program Offices
+• Ability to multi-task, organize and prioritize assignments
+• Production Experience and/or New Production Program Experience
+• Ability to construct PowerPoint presentation material and brief to senior leadership effectively
+• Active Top Secret security clearance
+Security Clearance Statement:This position requires a government security clearance, you must be a US Citizen for consideration.
+Clearance Level:Top Secret
+Other Important Information You Should Know
+Expression of Interest:By applying to this job, you are expressing interest in this position and could be considered for other career opportunities where similar skills and requirements have been identified as a match. Should this match be identified you may be contacted for this and future openings.
+Ability to Work Remotely:Onsite Full-time: The work associated with this position will be performed onsite at a designated Lockheed Martin facility.
+Work Schedules:Lockheed Martin supports a variety of alternate work schedules that provide additional flexibility to our employees. Schedules range from standard 40 hours over a five day work week while others may be condensed. These condensed schedules provide employees with additional time away from the office and are in addition to our Paid Time off benefits.
+Schedule for this Position:9x80 every other Friday off
+Pay Rate: The annual base salary range for this position in California and New York (excluding most major metropolitan areas), Colorado, Hawaii, Illinois, Maryland, Minnesota, New Jersey, Vermont, Washington or Washington DC is $77,700 - $136,965. For states not referenced above, the salary range for this position will reflect the candidate’s final work location. Please note that the salary information is a general guideline only. Lockheed Martin considers factors such as (but not limited to) scope and responsibilities of the position, candidate's work experience, education/ training, key skills as well as market and business considerations when extending an offer. Benefits offered: Medical, Dental, Vision, Life Insurance, Short-Term Disability, Long-Term Disability, 401(k) match, Flexible Spending Accounts, EAP, Education Assistance, Parental Leave, Paid time off, and Holidays. (Washington state applicants only) Non-represented full-time employees: accrue at least 10 hours per month of Paid Time Off (PTO) to be used for incidental absences and other reasons; receive at least 90 hours for holidays. Represented full time employees accrue 6.67 hours of Vacation per month; accrue up to 52 hours of sick leave annually; receive at least 96 hours for holidays. PTO, Vacation, sick leave, and holiday hours are prorated based on start date during the calendar year. This position is incentive plan eligible.
+Lockheed Martin is an equal opportunity employer. Qualified candidates will be considered without regard to legally protected characteristics.
+The application window will close in 90 days; applicants are encouraged to apply within 5 - 30 days of the requisition posting date in order to receive optimal consideration.
+At Lockheed Martin, we use our passion for purposeful innovation to help keep people safe and solve the world's most complex challenges. Our people are some of the greatest minds in the industry and truly make Lockheed Martin a great place to work.
+With our employees as our priority, we provide diverse career opportunities designed to propel, develop, and boost agility. Our flexible schedules, competitive pay, and comprehensive benefits enable our employees to live a healthy, fulfilling life at and outside of work. We place an emphasis on empowering our employees by fostering an inclusive environment built upon integrity and corporate responsibility.
+If this sounds like a culture you connect with, you’re invited to apply for this role. Or, if you are unsure whether your experience aligns with the requirements of this position, we encourage you to search on Lockheed Martin Jobs, and apply for roles that align with your qualifications.
+Experience Level:Experienced Professional
+Business Unit:SPACE
+Relocation Available:Possible
+Career Area:Manufacturing
+Type:Full-Time
+Shift:First</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr"/>
+      <c r="K4" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>